<commit_message>
update text with neew drafts
</commit_message>
<xml_diff>
--- a/inst/app/metadata/dmahler_2024-08-15.xlsx
+++ b/inst/app/metadata/dmahler_2024-08-15.xlsx
@@ -1,24 +1,98 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldbankgroup-my.sharepoint.com/personal/zprinsloo_worldbank_org/Documents/innovation_hub/InnovationHubDashboard/inst/app/metadata/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_EE78FDCE8F79A89360642C52EA5022B4917CBCE3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09ED4CE7-AFB7-4B77-A519-860B3B10D725}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="26370" yWindow="750" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>authors</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>paper_url</t>
+  </si>
+  <si>
+    <t>paper_publish_date</t>
+  </si>
+  <si>
+    <t>keywords</t>
+  </si>
+  <si>
+    <t>pip_vintage_primary_data</t>
+  </si>
+  <si>
+    <t>economy_excl_reason</t>
+  </si>
+  <si>
+    <t>aggregates_excl_reason</t>
+  </si>
+  <si>
+    <t>limitations</t>
+  </si>
+  <si>
+    <t>citation</t>
+  </si>
+  <si>
+    <t>Ending extreme poverty has a negligible impact on global greenhouse gas emissions</t>
+  </si>
+  <si>
+    <t>(Philip Wollburg, World Bank, pwollburg@worldbank.org); (Stephane Hallegatte, World Bank, shallegatte@worldbank.org); (Daniel Gerszon Mahler, World Bank, dmahler@worldbank.org)</t>
+  </si>
+  <si>
+    <t>The paper developed a method that converts income distributions to consumption distributions. The conversion relies on the modelled relationship between income and consumption distributions for countries that have both the same year.</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41586-023-06679-0</t>
+  </si>
+  <si>
+    <t>poverty; climate; emissions; inequality</t>
+  </si>
+  <si>
+    <t>20220909_2017_01_02_PROD</t>
+  </si>
+  <si>
+    <t>Economies using consumption are excluded because the purpose of the exercise was to convert income to consumption, so nothing was needed for those countries.</t>
+  </si>
+  <si>
+    <t>We did not compare aggregates using PIP's default estimates and our converted-consumption estimates because it wasn't central to the paper.</t>
+  </si>
+  <si>
+    <t>The method was tested on countries with both income and consumption estimates and extrapolated to countries with only income estimates. If these two types of countries differ, it is not guaranteed that the conversion works well for the countries we apply it to.</t>
+  </si>
+  <si>
+    <t>Wollburg, P., Hallegatte, S. &amp; Mahler, D.G. Ending extreme poverty has a negligible impact on global greenhouse gas emissions. Nature 623, 982–986 (2023). https://doi.org/10.1038/s41586-023-06679-0</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd HH:mm:ss UTC"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss\ \U\T\C"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -67,13 +141,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -111,7 +193,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -145,6 +227,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -179,9 +262,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -354,126 +438,87 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="20.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>authors</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>paper_url</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>paper_publish_date</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>keywords</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>pip_vintage_primary_data</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>economy_excl_reason</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>aggregates_excl_reason</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>limitations</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ending extreme poverty has a negligible impact on global greenhouse gas emissions</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>(Philip Wollburg, World Bank, pwollburg@worldbank.org); (Stephane Hallegatte, World Bank, shallegatte@worldbank.org); (Daniel Gerszon Mahler, World Bank, dmahler@worldbank.org)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>The paper developed a method that converts income distributions to consumption distributions. The conversion relies on the modelled relationship between income and consumption distributions for countries that have both the same year.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1038/s41586-023-06679-0</t>
-        </is>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
       </c>
       <c r="E2" s="2">
         <v>45259</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>poverty; climate; emissions; inequality</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>20220909_2017_01_02_PROD</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Economies using consumption are excluded because the purpose of the exercise was to convert income to consumption, so nothing was needed for those countries.</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>We did not compare aggregates using PIP's default estimates and our converted-consumption estimates because it wasn't central to the paper.</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>The method was tested on countries with both income and consumption estimates and extrapolated to countries with only income estimates. If these two types of countries differ, it is not guaranteed that the conversion works well for the countries we apply it to.</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Wollburg, P., Hallegatte, S. &amp; Mahler, D.G. Ending extreme poverty has a negligible impact on global greenhouse gas emissions. Nature 623, 982–986 (2023). https://doi.org/10.1038/s41586-023-06679-0</t>
-        </is>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;R_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Official Use Only</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>